<commit_message>
📊 BIST Screener | 01.05.2026 09:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-01.xlsx
+++ b/data/bist_screener_2026-05-01.xlsx
@@ -25744,48 +25744,58 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>80.53</v>
+        <v>5.68</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>0.0176</v>
+        <v>-0.0018</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>10440000</v>
-      </c>
-      <c r="E582" s="2" t="inlineStr"/>
+        <v>56180000</v>
+      </c>
+      <c r="E582" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F582" s="3" t="n">
-        <v>43.51</v>
+        <v>85.04000000000001</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
       <c r="I582" s="2" t="inlineStr"/>
       <c r="J582" s="2" t="inlineStr"/>
-      <c r="K582" s="2" t="inlineStr"/>
-      <c r="L582" s="2" t="inlineStr"/>
+      <c r="K582" s="2" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L582" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M582" s="2" t="inlineStr"/>
     </row>
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>40.58</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.0117</v>
-      </c>
-      <c r="D583" s="7" t="n">
-        <v>8380000.000000001</v>
+        <v>0.0071</v>
+      </c>
+      <c r="D583" s="9" t="n">
+        <v>255560</v>
       </c>
       <c r="E583" s="6" t="inlineStr"/>
       <c r="F583" s="7" t="n">
-        <v>54.32</v>
+        <v>11.8</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
@@ -25793,47 +25803,49 @@
       <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>21.46</v>
+        <v>17.94</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>0.0999</v>
+        <v>0.0022</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>86600000</v>
-      </c>
-      <c r="E584" s="2" t="inlineStr"/>
+        <v>1260000</v>
+      </c>
+      <c r="E584" s="4" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F584" s="3" t="n">
-        <v>68.67</v>
+        <v>58.1</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
-      <c r="I584" s="2" t="inlineStr"/>
-      <c r="J584" s="2" t="inlineStr"/>
+      <c r="I584" s="4" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J584" s="4" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25841,40 +25853,34 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>2.68</v>
+        <v>189.5</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0</v>
+        <v>0.0706</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>90400000</v>
-      </c>
-      <c r="E585" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>18010000</v>
+      </c>
+      <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>42.36</v>
+        <v>44.94</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J585" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I585" s="6" t="inlineStr"/>
+      <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25882,21 +25888,21 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>17.01</v>
+        <v>6.16</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0053</v>
+        <v>0.0016</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>72710000</v>
+        <v>7690000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>52.78</v>
+        <v>62.72</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25907,42 +25913,32 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L586" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="L586" s="2" t="inlineStr"/>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>ATAGY</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>13.16</v>
+        <v>2.94</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0273</v>
+        <v>0.09699999999999999</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>272910</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.6889</v>
-      </c>
+        <v>240000000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>56.17</v>
+        <v>55.79</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-0.0266</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-0.5014999999999999</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -25950,7 +25946,7 @@
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25958,34 +25954,42 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>162.5</v>
+        <v>17.05</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.0137</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>6940000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>11180000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>55.44</v>
-      </c>
-      <c r="G588" s="2" t="inlineStr"/>
+        <v>46.47</v>
+      </c>
+      <c r="G588" s="3" t="n">
+        <v>161.15</v>
+      </c>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25993,23 +25997,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>28.48</v>
+        <v>40.58</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0007000000000000001</v>
-      </c>
-      <c r="D589" s="9" t="n">
-        <v>18800000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>-0.0117</v>
+      </c>
+      <c r="D589" s="7" t="n">
+        <v>8380000.000000001</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>49.66</v>
+        <v>54.32</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26017,12 +26019,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26030,56 +26032,58 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>33.06</v>
+        <v>78.5</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0024</v>
+        <v>0.07980000000000001</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>4310000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>34400</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>48.1</v>
+        <v>43.41</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J590" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>6.16</v>
+        <v>162.5</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0016</v>
+        <v>0.0037</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>7690000</v>
+        <v>6940000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>62.72</v>
+        <v>55.44</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26087,41 +26091,39 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>17.94</v>
+        <v>17.01</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0022</v>
+        <v>-0.0053</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>1260000</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.9869</v>
-      </c>
+        <v>72710000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>58.1</v>
+        <v>52.78</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>0.3246</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26129,7 +26131,7 @@
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26137,38 +26139,40 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>65.34999999999999</v>
+        <v>7.62</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0106</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>665180</v>
+        <v>122010000</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.1672</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>58.93</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
       <c r="J593" s="8" t="n">
-        <v>0.4139</v>
+        <v>-4.2562</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26176,34 +26180,40 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>27.16</v>
+        <v>140.3</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0316</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>17070000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>2340000</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>63.67</v>
+        <v>46.39</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26248,75 +26258,67 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>19.01</v>
+        <v>80.53</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0031</v>
+        <v>0.0176</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>62410000</v>
+        <v>10440000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>29.07</v>
+        <v>43.51</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
       <c r="J596" s="2" t="inlineStr"/>
-      <c r="K596" s="2" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="K596" s="2" t="inlineStr"/>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>7.62</v>
+        <v>2.68</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>0</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>122010000</v>
+        <v>90400000</v>
       </c>
       <c r="E597" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.7119</v>
       </c>
       <c r="F597" s="7" t="n">
-        <v>70.51000000000001</v>
+        <v>42.36</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="8" t="n">
-        <v>-5.3262</v>
+        <v>-191.6342</v>
       </c>
       <c r="J597" s="8" t="n">
-        <v>-4.2562</v>
+        <v>-0.8093</v>
       </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26324,21 +26326,23 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>38.72</v>
+        <v>242</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0031</v>
+        <v>0</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>10070000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>7420</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>48.93</v>
+        <v>41.93</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26346,39 +26350,41 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr"/>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ATAGY</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>2.94</v>
+        <v>13.16</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.09699999999999999</v>
+        <v>-0.0273</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>240000000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>272910</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.6889</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>55.79</v>
+        <v>56.17</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="6" t="inlineStr"/>
+      <c r="I599" s="8" t="n">
+        <v>-0.0266</v>
+      </c>
+      <c r="J599" s="8" t="n">
+        <v>-0.5014999999999999</v>
+      </c>
       <c r="K599" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26386,7 +26392,7 @@
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26394,34 +26400,26 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>17.05</v>
+        <v>33.06</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0137</v>
+        <v>0.0024</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>11180000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>4310000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>46.47</v>
-      </c>
-      <c r="G600" s="3" t="n">
-        <v>161.15</v>
-      </c>
+        <v>48.1</v>
+      </c>
+      <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
           <t>Üretici imalatı</t>
@@ -26429,7 +26427,7 @@
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26472,21 +26470,21 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>92.09999999999999</v>
+        <v>38.72</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0071</v>
+        <v>0.0031</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>255560</v>
+        <v>10070000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>11.8</v>
+        <v>48.93</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26494,69 +26492,71 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>78.5</v>
+        <v>28.48</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.07980000000000001</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>34400</v>
+        <v>18800000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.58</v>
+        <v>0.2667</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>43.41</v>
+        <v>49.66</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>242</v>
+        <v>27.16</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>7420</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>17070000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>41.93</v>
+        <v>63.67</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26564,45 +26564,51 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr"/>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>5.68</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0018</v>
+        <v>-0.0106</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>56180000</v>
+        <v>665180</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>85.04000000000001</v>
+        <v>58.93</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="6" t="inlineStr"/>
+      <c r="J605" s="8" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26610,40 +26616,34 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>140.3</v>
+        <v>19.01</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0316</v>
+        <v>-0.0031</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>2340000</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>62410000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>46.39</v>
+        <v>29.07</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26651,21 +26651,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>189.5</v>
+        <v>21.46</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0706</v>
+        <v>0.0999</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>18010000</v>
+        <v>86600000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>44.94</v>
+        <v>68.67</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26673,12 +26673,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26705,7 +26705,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>01.05.2026 08:30</t>
+          <t>01.05.2026 09:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 01.05.2026 11:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-01.xlsx
+++ b/data/bist_screener_2026-05-01.xlsx
@@ -25787,38 +25787,34 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>65.34999999999999</v>
+        <v>27.16</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.0106</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>665180</v>
-      </c>
-      <c r="E583" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>17070000</v>
+      </c>
+      <c r="E583" s="6" t="inlineStr"/>
       <c r="F583" s="7" t="n">
-        <v>58.93</v>
+        <v>63.67</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
       <c r="I583" s="6" t="inlineStr"/>
-      <c r="J583" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L583" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M583" s="6" t="inlineStr"/>
@@ -25826,21 +25822,21 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>162.5</v>
+        <v>17.01</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>0.0037</v>
+        <v>-0.0053</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>6940000</v>
+        <v>72710000</v>
       </c>
       <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>55.44</v>
+        <v>52.78</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25848,12 +25844,12 @@
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25861,112 +25857,106 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>33.06</v>
+        <v>78.5</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0024</v>
+        <v>0.07980000000000001</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>4310000</v>
-      </c>
-      <c r="E585" s="6" t="inlineStr"/>
+        <v>34400</v>
+      </c>
+      <c r="E585" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F585" s="7" t="n">
-        <v>48.1</v>
+        <v>43.41</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="6" t="inlineStr"/>
-      <c r="J585" s="6" t="inlineStr"/>
+      <c r="I585" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J585" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L585" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L585" s="6" t="inlineStr"/>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>78.5</v>
+        <v>189.5</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.07980000000000001</v>
+        <v>0.0706</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>34400</v>
-      </c>
-      <c r="E586" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>18010000</v>
+      </c>
+      <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>43.41</v>
+        <v>44.94</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J586" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I586" s="2" t="inlineStr"/>
+      <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L586" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L586" s="2" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>7.62</v>
+        <v>21.46</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0999</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>122010000</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>86600000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>70.51000000000001</v>
+        <v>68.67</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25974,23 +25964,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>28.48</v>
+        <v>19.01</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0007000000000000001</v>
+        <v>-0.0031</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>18800000</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>62410000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>49.66</v>
+        <v>29.07</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25998,12 +25986,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -26011,23 +25999,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>242</v>
+        <v>33.06</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0</v>
+        <v>0.0024</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>7420</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>4310000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>41.93</v>
+        <v>48.1</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26035,32 +26021,34 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>5.68</v>
+        <v>13.98</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0018</v>
+        <v>0.0138</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>56180000</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>32400000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>85.04000000000001</v>
+        <v>54.25</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26068,12 +26056,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26081,34 +26069,40 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>13.98</v>
+        <v>17.94</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0138</v>
+        <v>0.0022</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>32400000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>1260000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>54.25</v>
+        <v>58.1</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26116,40 +26110,34 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>2.68</v>
+        <v>162.5</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0</v>
+        <v>0.0037</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>90400000</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>6940000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>42.36</v>
+        <v>55.44</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26157,34 +26145,42 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>2.94</v>
+        <v>17.05</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.09699999999999999</v>
+        <v>0.0137</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>240000000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>11180000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>55.79</v>
-      </c>
-      <c r="G593" s="6" t="inlineStr"/>
+        <v>46.47</v>
+      </c>
+      <c r="G593" s="7" t="n">
+        <v>161.15</v>
+      </c>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26192,21 +26188,21 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>21.46</v>
+        <v>2.94</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0999</v>
+        <v>0.09699999999999999</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>86600000</v>
+        <v>240000000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>68.67</v>
+        <v>55.79</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26214,12 +26210,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26227,122 +26223,124 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>189.5</v>
+        <v>7</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0706</v>
+        <v>-0.0182</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>18010000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>542950</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>44.94</v>
+        <v>37.31</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr"/>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>6.16</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0016</v>
+        <v>-0.0106</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>7690000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>665180</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>62.72</v>
+        <v>58.93</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="J596" s="4" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>19.01</v>
+        <v>80.53</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0031</v>
+        <v>0.0176</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>62410000</v>
+        <v>10440000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>29.07</v>
+        <v>43.51</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="6" t="inlineStr"/>
       <c r="J597" s="6" t="inlineStr"/>
-      <c r="K597" s="6" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="K597" s="6" t="inlineStr"/>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>40.58</v>
+        <v>6.16</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0117</v>
-      </c>
-      <c r="D598" s="3" t="n">
-        <v>8380000.000000001</v>
+        <v>0.0016</v>
+      </c>
+      <c r="D598" s="5" t="n">
+        <v>7690000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>54.32</v>
+        <v>62.72</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26350,61 +26348,67 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr"/>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>80.53</v>
+        <v>28.48</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0176</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>10440000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>18800000</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>43.51</v>
+        <v>49.66</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
       <c r="J599" s="6" t="inlineStr"/>
-      <c r="K599" s="6" t="inlineStr"/>
-      <c r="L599" s="6" t="inlineStr"/>
+      <c r="K599" s="6" t="inlineStr">
+        <is>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>27.16</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0071</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>17070000</v>
+        <v>255560</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>63.67</v>
+        <v>11.8</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26412,47 +26416,49 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr"/>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>17.01</v>
+        <v>2.68</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0053</v>
+        <v>0</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>72710000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>90400000</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>52.78</v>
+        <v>42.36</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26460,40 +26466,34 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>17.94</v>
+        <v>40.58</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0022</v>
-      </c>
-      <c r="D602" s="5" t="n">
-        <v>1260000</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.9869</v>
-      </c>
+        <v>-0.0117</v>
+      </c>
+      <c r="D602" s="3" t="n">
+        <v>8380000.000000001</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>58.1</v>
+        <v>54.32</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J602" s="4" t="n">
-        <v>0.3246</v>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
+      <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26501,21 +26501,23 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>92.09999999999999</v>
+        <v>5.68</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0071</v>
+        <v>-0.0018</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>255560</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>56180000</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>11.8</v>
+        <v>85.04000000000001</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26526,27 +26528,33 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L603" s="6" t="inlineStr"/>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>38.72</v>
+        <v>242</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0031</v>
+        <v>0</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>10070000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>7420</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>48.93</v>
+        <v>41.93</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26554,55 +26562,49 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr"/>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>17.05</v>
+        <v>140.3</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0137</v>
+        <v>0.0316</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>11180000</v>
+        <v>2340000</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.9246</v>
+        <v>0.1071</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>46.47</v>
-      </c>
-      <c r="G605" s="7" t="n">
-        <v>161.15</v>
-      </c>
+        <v>46.39</v>
+      </c>
+      <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="8" t="n">
-        <v>0.0028</v>
+        <v>-3.6635</v>
       </c>
       <c r="J605" s="8" t="n">
-        <v>-10.3171</v>
+        <v>-0.4897</v>
       </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26610,40 +26612,34 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>140.3</v>
+        <v>38.72</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0316</v>
+        <v>0.0031</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>2340000</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>10070000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>46.39</v>
+        <v>48.93</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26651,38 +26647,42 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>7</v>
+        <v>7.62</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0182</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>542950</v>
+        <v>122010000</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.95</v>
+        <v>0.1672</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>37.31</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
       <c r="I607" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-5.3262</v>
       </c>
       <c r="J607" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-4.2562</v>
       </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26707,7 +26707,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>01.05.2026 10:30</t>
+          <t>01.05.2026 11:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 01.05.2026 12:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-01.xlsx
+++ b/data/bist_screener_2026-05-01.xlsx
@@ -25787,34 +25787,40 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>27.16</v>
+        <v>2.68</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>0</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>17070000</v>
-      </c>
-      <c r="E583" s="6" t="inlineStr"/>
+        <v>90400000</v>
+      </c>
+      <c r="E583" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F583" s="7" t="n">
-        <v>63.67</v>
+        <v>42.36</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="6" t="inlineStr"/>
-      <c r="J583" s="6" t="inlineStr"/>
+      <c r="I583" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J583" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L583" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M583" s="6" t="inlineStr"/>
@@ -25822,34 +25828,38 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>17.01</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0053</v>
+        <v>-0.0106</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>72710000</v>
-      </c>
-      <c r="E584" s="2" t="inlineStr"/>
+        <v>665180</v>
+      </c>
+      <c r="E584" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F584" s="3" t="n">
-        <v>52.78</v>
+        <v>58.93</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="2" t="inlineStr"/>
-      <c r="J584" s="2" t="inlineStr"/>
+      <c r="J584" s="4" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25857,58 +25867,64 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>78.5</v>
+        <v>17.05</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.07980000000000001</v>
+        <v>0.0137</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>34400</v>
+        <v>11180000</v>
       </c>
       <c r="E585" s="8" t="n">
-        <v>0.58</v>
+        <v>0.9246</v>
       </c>
       <c r="F585" s="7" t="n">
-        <v>43.41</v>
-      </c>
-      <c r="G585" s="6" t="inlineStr"/>
+        <v>46.47</v>
+      </c>
+      <c r="G585" s="7" t="n">
+        <v>161.15</v>
+      </c>
       <c r="H585" s="6" t="inlineStr"/>
       <c r="I585" s="8" t="n">
-        <v>-9.409700000000001</v>
+        <v>0.0028</v>
       </c>
       <c r="J585" s="8" t="n">
-        <v>-4.155</v>
+        <v>-10.3171</v>
       </c>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L585" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L585" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+        </is>
+      </c>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>189.5</v>
+        <v>162.5</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0706</v>
+        <v>0.0037</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>18010000</v>
+        <v>6940000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>44.94</v>
+        <v>55.44</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25916,12 +25932,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25929,56 +25945,60 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>21.46</v>
+        <v>78.5</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0999</v>
+        <v>0.07980000000000001</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>86600000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>34400</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>68.67</v>
+        <v>43.41</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="I587" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J587" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr"/>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>19.01</v>
+        <v>5.68</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0031</v>
+        <v>-0.0018</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>62410000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>56180000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>29.07</v>
+        <v>85.04000000000001</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25991,7 +26011,7 @@
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25999,21 +26019,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>33.06</v>
+        <v>6.16</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0024</v>
+        <v>0.0016</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>4310000</v>
+        <v>7690000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>48.1</v>
+        <v>62.72</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26021,14 +26041,10 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
@@ -26069,62 +26085,48 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>17.94</v>
+        <v>80.53</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0022</v>
+        <v>0.0176</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>1260000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.9869</v>
-      </c>
+        <v>10440000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>58.1</v>
+        <v>43.51</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>0.3246</v>
-      </c>
-      <c r="K591" s="6" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST MENKUL KIYM YO</t>
-        </is>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
+      <c r="K591" s="6" t="inlineStr"/>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>162.5</v>
+        <v>17.01</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0037</v>
+        <v>-0.0053</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>6940000</v>
+        <v>72710000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>55.44</v>
+        <v>52.78</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26132,12 +26134,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26145,42 +26147,34 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>17.05</v>
+        <v>2.94</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0137</v>
+        <v>0.09699999999999999</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>11180000</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>240000000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>46.47</v>
-      </c>
-      <c r="G593" s="7" t="n">
-        <v>161.15</v>
-      </c>
+        <v>55.79</v>
+      </c>
+      <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J593" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26188,21 +26182,23 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>2.94</v>
+        <v>242</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.09699999999999999</v>
+        <v>0</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>240000000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>7420</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>55.79</v>
+        <v>41.93</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26210,88 +26206,90 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>7</v>
+        <v>17.94</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0182</v>
+        <v>0.0022</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>542950</v>
+        <v>1260000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.95</v>
+        <v>0.9869</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>37.31</v>
+        <v>58.1</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-0.2446</v>
       </c>
       <c r="J595" s="8" t="n">
-        <v>-0.4678</v>
+        <v>0.3246</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST MENKUL KIYM YO</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>65.34999999999999</v>
+        <v>7.62</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0106</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>665180</v>
+        <v>122010000</v>
       </c>
       <c r="E596" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.1672</v>
       </c>
       <c r="F596" s="3" t="n">
-        <v>58.93</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
       <c r="J596" s="4" t="n">
-        <v>0.4139</v>
+        <v>-4.2562</v>
       </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26299,48 +26297,62 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>80.53</v>
+        <v>140.3</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0176</v>
+        <v>0.0316</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>10440000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>2340000</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>43.51</v>
+        <v>46.39</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
-      <c r="K597" s="6" t="inlineStr"/>
-      <c r="L597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
+      <c r="K597" s="6" t="inlineStr">
+        <is>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>6.16</v>
+        <v>189.5</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0016</v>
+        <v>0.0706</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>7690000</v>
+        <v>18010000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>62.72</v>
+        <v>44.94</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26348,32 +26360,34 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>28.48</v>
+        <v>38.72</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0007000000000000001</v>
+        <v>0.0031</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>18800000</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>10070000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>49.66</v>
+        <v>48.93</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26381,12 +26395,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26425,40 +26439,36 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>2.68</v>
+        <v>28.48</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>90400000</v>
+        <v>18800000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.7119</v>
+        <v>0.2667</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>42.36</v>
+        <v>49.66</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26501,23 +26511,21 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>5.68</v>
+        <v>19.01</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0018</v>
+        <v>-0.0031</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>56180000</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>62410000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>85.04000000000001</v>
+        <v>29.07</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26530,7 +26538,7 @@
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26538,28 +26546,32 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>242</v>
+        <v>7</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0</v>
+        <v>-0.0182</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>7420</v>
+        <v>542950</v>
       </c>
       <c r="E604" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.95</v>
       </c>
       <c r="F604" s="3" t="n">
-        <v>41.93</v>
+        <v>37.31</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J604" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
           <t>İşlenebilen endüstriler</t>
@@ -26571,40 +26583,34 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>140.3</v>
+        <v>33.06</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0316</v>
+        <v>0.0024</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>2340000</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>4310000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>46.39</v>
+        <v>48.1</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26612,21 +26618,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>38.72</v>
+        <v>27.16</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0031</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>10070000</v>
+        <v>17070000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>48.93</v>
+        <v>63.67</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26634,12 +26640,12 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26647,40 +26653,34 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>7.62</v>
+        <v>21.46</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0999</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>122010000</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>86600000</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>70.51000000000001</v>
+        <v>68.67</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26707,7 +26707,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>01.05.2026 11:30</t>
+          <t>01.05.2026 12:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 01.05.2026 13:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-01.xlsx
+++ b/data/bist_screener_2026-05-01.xlsx
@@ -25787,40 +25787,36 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>2.68</v>
+        <v>5.68</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0</v>
+        <v>-0.0018</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>90400000</v>
+        <v>56180000</v>
       </c>
       <c r="E583" s="8" t="n">
-        <v>0.7119</v>
+        <v>0.8667</v>
       </c>
       <c r="F583" s="7" t="n">
-        <v>42.36</v>
+        <v>85.04000000000001</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J583" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I583" s="6" t="inlineStr"/>
+      <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L583" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M583" s="6" t="inlineStr"/>
@@ -25828,81 +25824,69 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>65.34999999999999</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0106</v>
+        <v>0.0071</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>665180</v>
-      </c>
-      <c r="E584" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>255560</v>
+      </c>
+      <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>58.93</v>
+        <v>11.8</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="2" t="inlineStr"/>
-      <c r="J584" s="4" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L584" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L584" s="2" t="inlineStr"/>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>17.05</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0137</v>
+        <v>-0.0106</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>11180000</v>
+        <v>665180</v>
       </c>
       <c r="E585" s="8" t="n">
-        <v>0.9246</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F585" s="7" t="n">
-        <v>46.47</v>
-      </c>
-      <c r="G585" s="7" t="n">
-        <v>161.15</v>
-      </c>
+        <v>58.93</v>
+      </c>
+      <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="8" t="n">
-        <v>0.0028</v>
-      </c>
+      <c r="I585" s="6" t="inlineStr"/>
       <c r="J585" s="8" t="n">
-        <v>-10.3171</v>
+        <v>0.4139</v>
       </c>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25910,130 +25894,122 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>162.5</v>
+        <v>80.53</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.0176</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>6940000</v>
+        <v>10440000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>55.44</v>
+        <v>43.51</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
       <c r="I586" s="2" t="inlineStr"/>
       <c r="J586" s="2" t="inlineStr"/>
-      <c r="K586" s="2" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L586" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+      <c r="K586" s="2" t="inlineStr"/>
+      <c r="L586" s="2" t="inlineStr"/>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>78.5</v>
+        <v>17.01</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.07980000000000001</v>
+        <v>-0.0053</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>34400</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>72710000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>43.41</v>
+        <v>52.78</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>5.68</v>
+        <v>78.5</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0018</v>
+        <v>0.07980000000000001</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>56180000</v>
+        <v>34400</v>
       </c>
       <c r="E588" s="4" t="n">
-        <v>0.8667</v>
+        <v>0.58</v>
       </c>
       <c r="F588" s="3" t="n">
-        <v>85.04000000000001</v>
+        <v>43.41</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>6.16</v>
+        <v>28.48</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0016</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>7690000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>18800000</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>62.72</v>
+        <v>49.66</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26041,92 +26017,106 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>13.98</v>
+        <v>7</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0138</v>
+        <v>-0.0182</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>32400000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>542950</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>54.25</v>
+        <v>37.31</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J590" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
           <t>İşlenebilen endüstriler</t>
         </is>
       </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>80.53</v>
+        <v>2.94</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0176</v>
+        <v>0.09699999999999999</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>10440000</v>
+        <v>240000000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>43.51</v>
+        <v>55.79</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
       <c r="J591" s="6" t="inlineStr"/>
-      <c r="K591" s="6" t="inlineStr"/>
-      <c r="L591" s="6" t="inlineStr"/>
+      <c r="K591" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>17.01</v>
+        <v>21.46</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0053</v>
+        <v>0.0999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>72710000</v>
+        <v>86600000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>52.78</v>
+        <v>68.67</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26134,12 +26124,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26147,21 +26137,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>2.94</v>
+        <v>27.16</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.09699999999999999</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>240000000</v>
+        <v>17070000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>55.79</v>
+        <v>63.67</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26169,12 +26159,12 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26182,23 +26172,21 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>242</v>
+        <v>40.58</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D594" s="5" t="n">
-        <v>7420</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>-0.0117</v>
+      </c>
+      <c r="D594" s="3" t="n">
+        <v>8380000.000000001</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>41.93</v>
+        <v>54.32</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26206,49 +26194,55 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>17.94</v>
+        <v>17.05</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0022</v>
+        <v>0.0137</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>1260000</v>
+        <v>11180000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.9869</v>
+        <v>0.9246</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>58.1</v>
-      </c>
-      <c r="G595" s="6" t="inlineStr"/>
+        <v>46.47</v>
+      </c>
+      <c r="G595" s="7" t="n">
+        <v>161.15</v>
+      </c>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="8" t="n">
-        <v>-0.2446</v>
+        <v>0.0028</v>
       </c>
       <c r="J595" s="8" t="n">
-        <v>0.3246</v>
+        <v>-10.3171</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26256,40 +26250,34 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>7.62</v>
+        <v>162.5</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0037</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>122010000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>6940000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>70.51000000000001</v>
+        <v>55.44</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26297,40 +26285,34 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>140.3</v>
+        <v>13.98</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0316</v>
+        <v>0.0138</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>2340000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>32400000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>46.39</v>
+        <v>54.25</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26338,21 +26320,21 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>189.5</v>
+        <v>38.72</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0706</v>
+        <v>0.0031</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>18010000</v>
+        <v>10070000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>44.94</v>
+        <v>48.93</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26360,12 +26342,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26373,34 +26355,40 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>38.72</v>
+        <v>17.94</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0031</v>
+        <v>0.0022</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>10070000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>1260000</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>48.93</v>
+        <v>58.1</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="6" t="inlineStr"/>
+      <c r="I599" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J599" s="8" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26408,21 +26396,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>92.09999999999999</v>
+        <v>19.01</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0071</v>
+        <v>-0.0031</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>255560</v>
+        <v>62410000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>11.8</v>
+        <v>29.07</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26433,42 +26421,50 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L600" s="2" t="inlineStr"/>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>28.48</v>
+        <v>7.62</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0007000000000000001</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>18800000</v>
+        <v>122010000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.1672</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>49.66</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26476,34 +26472,40 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>40.58</v>
+        <v>2.68</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0117</v>
-      </c>
-      <c r="D602" s="3" t="n">
-        <v>8380000.000000001</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D602" s="5" t="n">
+        <v>90400000</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>54.32</v>
+        <v>42.36</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
+      <c r="I602" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J602" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26511,21 +26513,23 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>19.01</v>
+        <v>242</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0031</v>
+        <v>0</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>62410000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>7420</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>29.07</v>
+        <v>41.93</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26533,71 +26537,65 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>7</v>
+        <v>33.06</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0182</v>
+        <v>0.0024</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>542950</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>4310000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>37.31</v>
+        <v>48.1</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>33.06</v>
+        <v>6.16</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0024</v>
+        <v>0.0016</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>4310000</v>
+        <v>7690000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>48.1</v>
+        <v>62.72</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26605,47 +26603,49 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>27.16</v>
+        <v>140.3</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0316</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>17070000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>2340000</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>63.67</v>
+        <v>46.39</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J606" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26653,21 +26653,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>21.46</v>
+        <v>189.5</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0999</v>
+        <v>0.0706</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>86600000</v>
+        <v>18010000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>68.67</v>
+        <v>44.94</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26675,12 +26675,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26707,7 +26707,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>01.05.2026 12:30</t>
+          <t>01.05.2026 13:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 01.05.2026 14:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-01.xlsx
+++ b/data/bist_screener_2026-05-01.xlsx
@@ -25787,36 +25787,40 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>5.68</v>
+        <v>140.3</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.0018</v>
+        <v>0.0316</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>56180000</v>
+        <v>2340000</v>
       </c>
       <c r="E583" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.1071</v>
       </c>
       <c r="F583" s="7" t="n">
-        <v>85.04000000000001</v>
+        <v>46.39</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="6" t="inlineStr"/>
-      <c r="J583" s="6" t="inlineStr"/>
+      <c r="I583" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J583" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L583" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M583" s="6" t="inlineStr"/>
@@ -25824,69 +25828,75 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>92.09999999999999</v>
+        <v>7.62</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>0.0071</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>255560</v>
-      </c>
-      <c r="E584" s="2" t="inlineStr"/>
+        <v>122010000</v>
+      </c>
+      <c r="E584" s="4" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F584" s="3" t="n">
-        <v>11.8</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
-      <c r="I584" s="2" t="inlineStr"/>
-      <c r="J584" s="2" t="inlineStr"/>
+      <c r="I584" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J584" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K584" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
         </is>
       </c>
-      <c r="L584" s="2" t="inlineStr"/>
+      <c r="L584" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>65.34999999999999</v>
+        <v>27.16</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.0106</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>665180</v>
-      </c>
-      <c r="E585" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>17070000</v>
+      </c>
+      <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>58.93</v>
+        <v>63.67</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
       <c r="I585" s="6" t="inlineStr"/>
-      <c r="J585" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25921,21 +25931,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>17.01</v>
+        <v>19.01</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0053</v>
+        <v>-0.0031</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>72710000</v>
+        <v>62410000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>52.78</v>
+        <v>29.07</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25948,7 +25958,7 @@
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25956,73 +25966,75 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>78.5</v>
+        <v>17.01</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.07980000000000001</v>
+        <v>-0.0053</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>34400</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>72710000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>43.41</v>
+        <v>52.78</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J588" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>28.48</v>
+        <v>17.94</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0007000000000000001</v>
+        <v>0.0022</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>18800000</v>
+        <v>1260000</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.9869</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>49.66</v>
+        <v>58.1</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="I589" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J589" s="8" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26030,35 +26042,29 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>7</v>
+        <v>6.16</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0182</v>
+        <v>0.0016</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>542950</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>7690000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>37.31</v>
+        <v>62.72</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J590" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I590" s="2" t="inlineStr"/>
+      <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr"/>
@@ -26067,36 +26073,38 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>2.94</v>
+        <v>7</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.09699999999999999</v>
+        <v>-0.0182</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>240000000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>542950</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>55.79</v>
+        <v>37.31</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
@@ -26137,21 +26145,23 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>27.16</v>
+        <v>28.48</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>17070000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>18800000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>63.67</v>
+        <v>49.66</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26159,12 +26169,12 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26207,42 +26217,34 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>17.05</v>
+        <v>162.5</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0137</v>
+        <v>0.0037</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>11180000</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>6940000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>46.47</v>
-      </c>
-      <c r="G595" s="7" t="n">
-        <v>161.15</v>
-      </c>
+        <v>55.44</v>
+      </c>
+      <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J595" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26250,21 +26252,21 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>162.5</v>
+        <v>13.98</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.0138</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>6940000</v>
+        <v>32400000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>55.44</v>
+        <v>54.25</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26272,12 +26274,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26285,21 +26287,23 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>13.98</v>
+        <v>5.68</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0138</v>
+        <v>-0.0018</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>32400000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>56180000</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>54.25</v>
+        <v>85.04000000000001</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26307,12 +26311,12 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26355,40 +26359,34 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>17.94</v>
+        <v>33.06</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0022</v>
+        <v>0.0024</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>1260000</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.9869</v>
-      </c>
+        <v>4310000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>58.1</v>
+        <v>48.1</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="8" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J599" s="8" t="n">
-        <v>0.3246</v>
-      </c>
+      <c r="I599" s="6" t="inlineStr"/>
+      <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26396,21 +26394,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>19.01</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0031</v>
+        <v>0.0071</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>62410000</v>
+        <v>255560</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>29.07</v>
+        <v>11.8</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26421,52 +26419,40 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L600" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="L600" s="2" t="inlineStr"/>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>7.62</v>
+        <v>242</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>0</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>122010000</v>
+        <v>7420</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.2578</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>70.51000000000001</v>
+        <v>41.93</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
@@ -26513,54 +26499,64 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>242</v>
+        <v>17.05</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0</v>
+        <v>0.0137</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>7420</v>
+        <v>11180000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.9246</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>41.93</v>
-      </c>
-      <c r="G603" s="6" t="inlineStr"/>
+        <v>46.47</v>
+      </c>
+      <c r="G603" s="7" t="n">
+        <v>161.15</v>
+      </c>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>33.06</v>
+        <v>189.5</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0024</v>
+        <v>0.0706</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>4310000</v>
+        <v>18010000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>48.1</v>
+        <v>44.94</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26568,12 +26564,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26581,93 +26577,97 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>6.16</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0016</v>
+        <v>-0.0106</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>7690000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>665180</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>62.72</v>
+        <v>58.93</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="6" t="inlineStr"/>
+      <c r="J605" s="8" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>140.3</v>
+        <v>78.5</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0316</v>
+        <v>0.07980000000000001</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>2340000</v>
+        <v>34400</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.58</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>46.39</v>
+        <v>43.41</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="4" t="n">
-        <v>-3.6635</v>
+        <v>-9.409700000000001</v>
       </c>
       <c r="J606" s="4" t="n">
-        <v>-0.4897</v>
+        <v>-4.155</v>
       </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>189.5</v>
+        <v>2.94</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0706</v>
+        <v>0.09699999999999999</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>18010000</v>
+        <v>240000000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>44.94</v>
+        <v>55.79</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26675,12 +26675,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26707,7 +26707,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>01.05.2026 13:30</t>
+          <t>01.05.2026 14:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 01.05.2026 15:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-01.xlsx
+++ b/data/bist_screener_2026-05-01.xlsx
@@ -25787,81 +25787,67 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>140.3</v>
+        <v>242</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0316</v>
+        <v>0</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>2340000</v>
+        <v>7420</v>
       </c>
       <c r="E583" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.2578</v>
       </c>
       <c r="F583" s="7" t="n">
-        <v>46.39</v>
+        <v>41.93</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J583" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I583" s="6" t="inlineStr"/>
+      <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>7.62</v>
+        <v>40.58</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>0.09960000000000001</v>
-      </c>
-      <c r="D584" s="5" t="n">
-        <v>122010000</v>
-      </c>
-      <c r="E584" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>-0.0117</v>
+      </c>
+      <c r="D584" s="3" t="n">
+        <v>8380000.000000001</v>
+      </c>
+      <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>70.51000000000001</v>
+        <v>54.32</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
-      <c r="I584" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J584" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I584" s="2" t="inlineStr"/>
+      <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25869,21 +25855,21 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>27.16</v>
+        <v>6.16</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0016</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>17070000</v>
+        <v>7690000</v>
       </c>
       <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>63.67</v>
+        <v>62.72</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25891,61 +25877,65 @@
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L585" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L585" s="6" t="inlineStr"/>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>80.53</v>
+        <v>27.16</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0176</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>10440000</v>
+        <v>17070000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>43.51</v>
+        <v>63.67</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
       <c r="I586" s="2" t="inlineStr"/>
       <c r="J586" s="2" t="inlineStr"/>
-      <c r="K586" s="2" t="inlineStr"/>
-      <c r="L586" s="2" t="inlineStr"/>
+      <c r="K586" s="2" t="inlineStr">
+        <is>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L586" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>19.01</v>
+        <v>17.01</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0031</v>
+        <v>-0.0053</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>62410000</v>
+        <v>72710000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>29.07</v>
+        <v>52.78</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25958,7 +25948,7 @@
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25966,21 +25956,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>17.01</v>
+        <v>21.46</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0053</v>
+        <v>0.0999</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>72710000</v>
+        <v>86600000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>52.78</v>
+        <v>68.67</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25988,12 +25978,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -26001,31 +25991,31 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>17.94</v>
+        <v>7.62</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0022</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>1260000</v>
+        <v>122010000</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.9869</v>
+        <v>0.1672</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>58.1</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="8" t="n">
-        <v>-0.2446</v>
+        <v>-5.3262</v>
       </c>
       <c r="J589" s="8" t="n">
-        <v>0.3246</v>
+        <v>-4.2562</v>
       </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
@@ -26034,7 +26024,7 @@
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26042,21 +26032,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>6.16</v>
+        <v>19.01</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0016</v>
+        <v>-0.0031</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>7690000</v>
+        <v>62410000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>62.72</v>
+        <v>29.07</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26067,101 +26057,103 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L590" s="2" t="inlineStr"/>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>7</v>
+        <v>162.5</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0182</v>
+        <v>0.0037</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>542950</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>6940000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>37.31</v>
+        <v>55.44</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>21.46</v>
+        <v>7</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0999</v>
+        <v>-0.0182</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>86600000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>542950</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>68.67</v>
+        <v>37.31</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J592" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>28.48</v>
+        <v>38.72</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0007000000000000001</v>
+        <v>0.0031</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>18800000</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>10070000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>49.66</v>
+        <v>48.93</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26169,12 +26161,12 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26182,21 +26174,23 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>40.58</v>
+        <v>5.68</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0117</v>
-      </c>
-      <c r="D594" s="3" t="n">
-        <v>8380000.000000001</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>-0.0018</v>
+      </c>
+      <c r="D594" s="5" t="n">
+        <v>56180000</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>54.32</v>
+        <v>85.04000000000001</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26204,12 +26198,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26217,21 +26211,23 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>162.5</v>
+        <v>28.48</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0037</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>6940000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>18800000</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>55.44</v>
+        <v>49.66</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26239,12 +26235,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26287,23 +26283,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>5.68</v>
+        <v>33.06</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0018</v>
+        <v>0.0024</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>56180000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>4310000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>85.04000000000001</v>
+        <v>48.1</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26311,12 +26305,12 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26324,34 +26318,40 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>38.72</v>
+        <v>140.3</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0031</v>
+        <v>0.0316</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>10070000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>2340000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>48.93</v>
+        <v>46.39</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J598" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26359,34 +26359,40 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>33.06</v>
+        <v>2.68</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0024</v>
+        <v>0</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>4310000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>90400000</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>48.1</v>
+        <v>42.36</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="6" t="inlineStr"/>
+      <c r="I599" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J599" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26394,21 +26400,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>92.09999999999999</v>
+        <v>2.94</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0071</v>
+        <v>0.09699999999999999</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>255560</v>
+        <v>240000000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>11.8</v>
+        <v>55.79</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26419,29 +26425,31 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L600" s="2" t="inlineStr"/>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>242</v>
+        <v>189.5</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0</v>
+        <v>0.0706</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>7420</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>18010000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>41.93</v>
+        <v>44.94</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26449,49 +26457,55 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>2.68</v>
+        <v>17.05</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0</v>
+        <v>0.0137</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>90400000</v>
+        <v>11180000</v>
       </c>
       <c r="E602" s="4" t="n">
-        <v>0.7119</v>
+        <v>0.9246</v>
       </c>
       <c r="F602" s="3" t="n">
-        <v>42.36</v>
-      </c>
-      <c r="G602" s="2" t="inlineStr"/>
+        <v>46.47</v>
+      </c>
+      <c r="G602" s="3" t="n">
+        <v>161.15</v>
+      </c>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="4" t="n">
-        <v>-191.6342</v>
+        <v>0.0028</v>
       </c>
       <c r="J602" s="4" t="n">
-        <v>-0.8093</v>
+        <v>-10.3171</v>
       </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26499,64 +26513,48 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>17.05</v>
+        <v>80.53</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0137</v>
+        <v>0.0176</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>11180000</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>10440000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>46.47</v>
-      </c>
-      <c r="G603" s="7" t="n">
-        <v>161.15</v>
-      </c>
+        <v>43.51</v>
+      </c>
+      <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
-      <c r="K603" s="6" t="inlineStr">
-        <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
+      <c r="K603" s="6" t="inlineStr"/>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>189.5</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0706</v>
+        <v>0.0071</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>18010000</v>
+        <v>255560</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>44.94</v>
+        <v>11.8</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26564,51 +26562,49 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr"/>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>65.34999999999999</v>
+        <v>17.94</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0106</v>
+        <v>0.0022</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>665180</v>
+        <v>1260000</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.9869</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>58.93</v>
+        <v>58.1</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="6" t="inlineStr"/>
+      <c r="I605" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
       <c r="J605" s="8" t="n">
-        <v>0.4139</v>
+        <v>0.3246</v>
       </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26616,73 +26612,77 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>78.5</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.07980000000000001</v>
+        <v>-0.0106</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>34400</v>
+        <v>665180</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.58</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>43.41</v>
+        <v>58.93</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
       <c r="J606" s="4" t="n">
-        <v>-4.155</v>
+        <v>0.4139</v>
       </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>2.94</v>
+        <v>78.5</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.09699999999999999</v>
+        <v>0.07980000000000001</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>240000000</v>
-      </c>
-      <c r="E607" s="6" t="inlineStr"/>
+        <v>34400</v>
+      </c>
+      <c r="E607" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F607" s="7" t="n">
-        <v>55.79</v>
+        <v>43.41</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="6" t="inlineStr"/>
-      <c r="J607" s="6" t="inlineStr"/>
+      <c r="I607" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J607" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26707,7 +26707,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>01.05.2026 14:30</t>
+          <t>01.05.2026 15:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 01.05.2026 16:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-01.xlsx
+++ b/data/bist_screener_2026-05-01.xlsx
@@ -25787,23 +25787,21 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>242</v>
+        <v>40.58</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D583" s="9" t="n">
-        <v>7420</v>
-      </c>
-      <c r="E583" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>-0.0117</v>
+      </c>
+      <c r="D583" s="7" t="n">
+        <v>8380000.000000001</v>
+      </c>
+      <c r="E583" s="6" t="inlineStr"/>
       <c r="F583" s="7" t="n">
-        <v>41.93</v>
+        <v>54.32</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
@@ -25811,30 +25809,34 @@
       <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>40.58</v>
+        <v>38.72</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0117</v>
-      </c>
-      <c r="D584" s="3" t="n">
-        <v>8380000.000000001</v>
+        <v>0.0031</v>
+      </c>
+      <c r="D584" s="5" t="n">
+        <v>10070000</v>
       </c>
       <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>54.32</v>
+        <v>48.93</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25842,12 +25844,12 @@
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25855,21 +25857,21 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>6.16</v>
+        <v>189.5</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0016</v>
+        <v>0.0706</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>7690000</v>
+        <v>18010000</v>
       </c>
       <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>62.72</v>
+        <v>44.94</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25877,30 +25879,34 @@
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L585" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L585" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>27.16</v>
+        <v>19.01</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.0031</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>17070000</v>
+        <v>62410000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>63.67</v>
+        <v>29.07</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25908,12 +25914,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -26032,21 +26038,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>19.01</v>
+        <v>6.16</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0031</v>
+        <v>0.0016</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>62410000</v>
+        <v>7690000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>29.07</v>
+        <v>62.72</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26057,44 +26063,46 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>162.5</v>
+        <v>140.3</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0037</v>
+        <v>0.0316</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>6940000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>2340000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>55.44</v>
+        <v>46.39</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26102,32 +26110,28 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>7</v>
+        <v>242</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0182</v>
+        <v>0</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>542950</v>
+        <v>7420</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.95</v>
+        <v>0.2578</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>37.31</v>
+        <v>41.93</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
           <t>İşlenebilen endüstriler</t>
@@ -26139,21 +26143,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>38.72</v>
+        <v>162.5</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0031</v>
+        <v>0.0037</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>10070000</v>
+        <v>6940000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>48.93</v>
+        <v>55.44</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26161,7 +26165,7 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
@@ -26174,60 +26178,58 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>5.68</v>
+        <v>7</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0018</v>
+        <v>-0.0182</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>56180000</v>
+        <v>542950</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.8667</v>
+        <v>0.95</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>85.04000000000001</v>
+        <v>37.31</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>28.48</v>
+        <v>13.98</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0007000000000000001</v>
+        <v>0.0138</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>18800000</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>32400000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>49.66</v>
+        <v>54.25</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26235,12 +26237,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26248,34 +26250,40 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>13.98</v>
+        <v>2.68</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0138</v>
+        <v>0</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>32400000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>90400000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>54.25</v>
+        <v>42.36</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26283,34 +26291,40 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>33.06</v>
+        <v>17.94</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0024</v>
+        <v>0.0022</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>4310000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>1260000</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>48.1</v>
+        <v>58.1</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26318,40 +26332,34 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>140.3</v>
+        <v>2.94</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0316</v>
+        <v>0.09699999999999999</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>2340000</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>240000000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>46.39</v>
+        <v>55.79</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J598" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I598" s="2" t="inlineStr"/>
+      <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26359,40 +26367,38 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>2.68</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0</v>
+        <v>-0.0106</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>90400000</v>
+        <v>665180</v>
       </c>
       <c r="E599" s="8" t="n">
-        <v>0.7119</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F599" s="7" t="n">
-        <v>42.36</v>
+        <v>58.93</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I599" s="6" t="inlineStr"/>
       <c r="J599" s="8" t="n">
-        <v>-0.8093</v>
+        <v>0.4139</v>
       </c>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26400,56 +26406,48 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>2.94</v>
+        <v>80.53</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.09699999999999999</v>
+        <v>0.0176</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>240000000</v>
+        <v>10440000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>55.79</v>
+        <v>43.51</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
       <c r="J600" s="2" t="inlineStr"/>
-      <c r="K600" s="2" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="K600" s="2" t="inlineStr"/>
+      <c r="L600" s="2" t="inlineStr"/>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>189.5</v>
+        <v>27.16</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0706</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>18010000</v>
+        <v>17070000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>44.94</v>
+        <v>63.67</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26457,12 +26455,12 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26470,34 +26468,26 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>17.05</v>
+        <v>33.06</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0137</v>
+        <v>0.0024</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>11180000</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>4310000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>46.47</v>
-      </c>
-      <c r="G602" s="3" t="n">
-        <v>161.15</v>
-      </c>
+        <v>48.1</v>
+      </c>
+      <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J602" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
+      <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
           <t>Üretici imalatı</t>
@@ -26505,7 +26495,7 @@
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26513,98 +26503,116 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>80.53</v>
+        <v>78.5</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0176</v>
+        <v>0.07980000000000001</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>10440000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>34400</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>43.51</v>
+        <v>43.41</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
-      <c r="K603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-4.155</v>
+      </c>
+      <c r="K603" s="6" t="inlineStr">
+        <is>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
       <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>92.09999999999999</v>
+        <v>17.05</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0071</v>
+        <v>0.0137</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>255560</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>11180000</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="G604" s="2" t="inlineStr"/>
+        <v>46.47</v>
+      </c>
+      <c r="G604" s="3" t="n">
+        <v>161.15</v>
+      </c>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J604" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>17.94</v>
+        <v>28.48</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0022</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>1260000</v>
+        <v>18800000</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.9869</v>
+        <v>0.2667</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>58.1</v>
+        <v>49.66</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>0.3246</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26612,77 +26620,69 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>65.34999999999999</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0106</v>
+        <v>0.0071</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>665180</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>255560</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>58.93</v>
+        <v>11.8</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="4" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>78.5</v>
+        <v>5.68</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.07980000000000001</v>
+        <v>-0.0018</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>34400</v>
+        <v>56180000</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.58</v>
+        <v>0.8667</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>43.41</v>
+        <v>85.04000000000001</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26707,7 +26707,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>01.05.2026 15:30</t>
+          <t>01.05.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>